<commit_message>
Move stray data files to data/
</commit_message>
<xml_diff>
--- a/data/harga_saham_ihsg.xlsx
+++ b/data/harga_saham_ihsg.xlsx
@@ -55,7 +55,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -88,12 +88,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00dcfce7"/>
-        <bgColor rgb="00dcfce7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00fee2e2"/>
         <bgColor rgb="00fee2e2"/>
       </patternFill>
@@ -117,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -129,11 +123,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -568,28 +561,28 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>5853.95</v>
+        <v>5788.91</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>53.95</v>
+        <v>-11.09</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.92</v>
+        <v>-0.19</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>5881.93</v>
+        <v>5798.96</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>5827.34</v>
+        <v>5765.79</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>653M</t>
+          <t>657M</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -600,23 +593,23 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>5832.13</v>
+        <v>5776.74</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>11.55</v>
+        <v>1.51</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.2</v>
+        <v>0.03</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>5856.2</v>
+        <v>5781.7</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>5808.37</v>
+        <v>5747.07</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>765M</t>
+          <t>543M</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -632,28 +625,28 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>5821.56</v>
+        <v>5766.02</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>26.72</v>
+        <v>2.44</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.46</v>
+        <v>0.04</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>5832.08</v>
+        <v>5776.18</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5794.03</v>
+        <v>5739.38</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>570M</t>
+          <t>535M</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -664,28 +657,28 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>5865.62</v>
+        <v>5801.38</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>49.3</v>
+        <v>-25.52</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.84</v>
+        <v>-0.44</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5895.52</v>
+        <v>5812.02</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>5857.77</v>
+        <v>5780.75</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>722M</t>
+          <t>739M</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -696,28 +689,28 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>5830.65</v>
+        <v>5868.83</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>-41.44</v>
+        <v>15.72</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.71</v>
+        <v>0.27</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>5844.51</v>
+        <v>5879.8</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>5813</v>
+        <v>5843.9</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>718M</t>
+          <t>644M</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -728,28 +721,28 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>5843.69</v>
+        <v>5821.84</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>31.45</v>
+        <v>2.25</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.54</v>
+        <v>0.04</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>5860.6</v>
+        <v>5824.5</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>5817.83</v>
+        <v>5806.56</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>658M</t>
+          <t>710M</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -760,28 +753,28 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>5884.57</v>
+        <v>5855.93</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>44.28</v>
+        <v>-7.6</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.75</v>
+        <v>-0.13</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5909.94</v>
+        <v>5858.88</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5866.47</v>
+        <v>5842.84</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>688M</t>
+          <t>536M</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -792,23 +785,23 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>5847.09</v>
+        <v>5895.75</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>42.25</v>
+        <v>48.5</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.72</v>
+        <v>0.82</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5856.51</v>
+        <v>5914.06</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>5837</v>
+        <v>5891.38</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>751M</t>
+          <t>551M</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -824,28 +817,28 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>5803.35</v>
+        <v>5800.92</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>16.46</v>
+        <v>-48.34</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.28</v>
+        <v>-0.83</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>5815.82</v>
+        <v>5819.44</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>5802.01</v>
+        <v>5774.65</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>618M</t>
+          <t>706M</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -856,23 +849,23 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>5784.97</v>
+        <v>5881.46</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>-15.72</v>
+        <v>-10.36</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.27</v>
+        <v>-0.18</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5809.09</v>
+        <v>5902.5</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>5776.92</v>
+        <v>5866.58</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>661M</t>
+          <t>522M</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -888,23 +881,23 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>5828.02</v>
+        <v>5861.37</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>51.12</v>
+        <v>43.07</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.88</v>
+        <v>0.73</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5828.29</v>
+        <v>5870.29</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>5807.05</v>
+        <v>5832.24</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>629M</t>
+          <t>784M</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -920,28 +913,28 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>5852.11</v>
+        <v>5813.4</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>44.17</v>
+        <v>-44.42</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.75</v>
+        <v>-0.76</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>5867.72</v>
+        <v>5813.83</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>5826.91</v>
+        <v>5803.12</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>580M</t>
+          <t>543M</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -952,28 +945,28 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>5843.36</v>
+        <v>5761.2</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>-2.94</v>
+        <v>-40.38</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.05</v>
+        <v>-0.7</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>5868.9</v>
+        <v>5768.23</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>5824.95</v>
+        <v>5733.91</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>766M</t>
+          <t>603M</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -984,28 +977,28 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>5819.47</v>
+        <v>5917.93</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>43.12</v>
+        <v>-18.15</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.74</v>
+        <v>-0.31</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>5844.74</v>
+        <v>5927.21</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>5793.3</v>
+        <v>5888.94</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>695M</t>
+          <t>588M</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1016,23 +1009,23 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>5804.97</v>
+        <v>5971.99</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>40.95</v>
+        <v>30.78</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.71</v>
+        <v>0.52</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>5812.14</v>
+        <v>5988.79</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>5785.5</v>
+        <v>5952.73</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>699M</t>
+          <t>672M</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1048,23 +1041,23 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>5738.32</v>
+        <v>5820.73</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>-11.07</v>
+        <v>-18.34</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.32</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5748.15</v>
+        <v>5844.5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>5725.08</v>
+        <v>5807.07</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>685M</t>
+          <t>697M</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1080,28 +1073,28 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5805.16</v>
+        <v>5882.81</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>-32.16</v>
+        <v>43.16</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>-0.55</v>
+        <v>0.73</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>5815.26</v>
+        <v>5905.41</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>5784.27</v>
+        <v>5863.16</v>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>660M</t>
+          <t>580M</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1112,23 +1105,23 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>5841.96</v>
+        <v>5899.53</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>33.75</v>
+        <v>55.41</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.58</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>5854.48</v>
+        <v>5925.12</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>5838.08</v>
+        <v>5891.85</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>799M</t>
+          <t>735M</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1144,28 +1137,28 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>6089.53</v>
+        <v>5816.7</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>46.85</v>
+        <v>19.85</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.77</v>
+        <v>0.34</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>6096.59</v>
+        <v>5845.56</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>6081.29</v>
+        <v>5790.09</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>601M</t>
+          <t>689M</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1176,28 +1169,28 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>5796.46</v>
+        <v>5908.96</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>27.95</v>
+        <v>-42.91</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.48</v>
+        <v>-0.73</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>5801.46</v>
+        <v>5918.81</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>5773.53</v>
+        <v>5890.24</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>681M</t>
+          <t>780M</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1208,28 +1201,28 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>5786.44</v>
+        <v>5938.92</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>-36.94</v>
+        <v>28.65</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.64</v>
+        <v>0.48</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>5807.92</v>
+        <v>5945.81</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>5775.65</v>
+        <v>5913.81</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>563M</t>
+          <t>729M</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1240,23 +1233,23 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>5725.25</v>
+        <v>5721.81</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>-25.65</v>
+        <v>-36.49</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.45</v>
+        <v>-0.64</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>5728.71</v>
+        <v>5743.9</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>5700.24</v>
+        <v>5700.58</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>530M</t>
+          <t>776M</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1272,23 +1265,23 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>5904.82</v>
+        <v>5828.96</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>27.47</v>
+        <v>21.39</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.47</v>
+        <v>0.37</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>5924.2</v>
+        <v>5842</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5893.31</v>
+        <v>5809.84</v>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>606M</t>
+          <t>679M</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -1304,28 +1297,28 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>5825.24</v>
+        <v>5764.81</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>45.86</v>
+        <v>-6.37</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.79</v>
+        <v>-0.11</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>5832.43</v>
+        <v>5788.33</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>5813.66</v>
+        <v>5752.05</v>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>591M</t>
+          <t>728M</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1336,23 +1329,23 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>5936.75</v>
+        <v>5964.13</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>57.04</v>
+        <v>43.3</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.96</v>
+        <v>0.73</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>5945.81</v>
+        <v>5993.63</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>5908.81</v>
+        <v>5935.9</v>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>657M</t>
+          <t>751M</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -1368,28 +1361,28 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>5847.7</v>
+        <v>5761.85</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>-47.15</v>
+        <v>-18.51</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.32</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>5866.46</v>
+        <v>5780.05</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5837.95</v>
+        <v>5749.62</v>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>580M</t>
+          <t>681M</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1400,28 +1393,28 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>6199.7</v>
+        <v>5886.57</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>25.86</v>
+        <v>6.53</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.42</v>
+        <v>0.11</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>6201.41</v>
+        <v>5887.45</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>6182.14</v>
+        <v>5885.72</v>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>656M</t>
+          <t>524M</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1432,28 +1425,28 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>5947.57</v>
+        <v>5832.26</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>39.71</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.67</v>
+        <v>0.16</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>5969.15</v>
+        <v>5841.91</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>5944.09</v>
+        <v>5816</v>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>617M</t>
+          <t>609M</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1464,28 +1457,28 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>5879.33</v>
+        <v>5825.63</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>3.15</v>
+        <v>41.81</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0.05</v>
+        <v>0.72</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>5905.73</v>
+        <v>5851.21</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>5868.92</v>
+        <v>5824.49</v>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>594M</t>
+          <t>724M</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1496,28 +1489,28 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>5895.94</v>
+        <v>5870.92</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>-24.57</v>
+        <v>15.9</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.42</v>
+        <v>0.27</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>5906.78</v>
+        <v>5896.84</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>5884.55</v>
+        <v>5843.84</v>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>620M</t>
+          <t>563M</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1528,28 +1521,28 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>5802.61</v>
+        <v>5936.66</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>40.37</v>
+        <v>18.95</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.7</v>
+        <v>0.32</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>5803.45</v>
+        <v>5947.6</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>5788.06</v>
+        <v>5912.04</v>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>676M</t>
+          <t>640M</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -2078,16 +2071,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9900</v>
+        <v>10050</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>-1.03</v>
+        <v>1.58</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.01</v>
+        <v>0.02</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>46.1</v>
+        <v>47.6</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
@@ -2105,16 +2098,16 @@
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>11.8</v>
+        <v>11</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>14.7</v>
+        <v>13.7</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>842.35</v>
+        <v>917.05</v>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
@@ -2139,16 +2132,16 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>5450</v>
+        <v>4150</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1.21</v>
+        <v>-0.48</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.02</v>
+        <v>-0.01</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>53.1</v>
+        <v>40.1</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
@@ -2166,16 +2159,16 @@
         </is>
       </c>
       <c r="K3" s="3" t="n">
-        <v>13.1</v>
+        <v>12.5</v>
       </c>
       <c r="L3" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>16.4</v>
+        <v>15.6</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>414.64</v>
+        <v>333.19</v>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
@@ -2200,16 +2193,16 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3250</v>
+        <v>2900</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-1.3</v>
+        <v>-0.73</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>50.6</v>
+        <v>48.4</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -2227,16 +2220,16 @@
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>13.4</v>
+        <v>13.6</v>
       </c>
       <c r="L4" s="3" t="n">
         <v>2.4</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>16.2</v>
+        <v>16.6</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>243.35</v>
+        <v>212.65</v>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
@@ -2261,16 +2254,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5550</v>
+        <v>5750</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>3.35</v>
+        <v>-0.03</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.06</v>
+        <v>-0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>54.7</v>
+        <v>51.3</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -2288,16 +2281,16 @@
         </is>
       </c>
       <c r="K5" s="3" t="n">
-        <v>10.3</v>
+        <v>10.7</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>1.9</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>14.4</v>
+        <v>15</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>539.88</v>
+        <v>535.17</v>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
@@ -2322,16 +2315,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3600</v>
+        <v>3500</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-2.04</v>
+        <v>1.12</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.06</v>
+        <v>0.03</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>38.2</v>
+        <v>45.5</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -2349,16 +2342,16 @@
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>22.8</v>
+        <v>25.6</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3.6</v>
+        <v>4.1</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>16.4</v>
+        <v>18.5</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>157.94</v>
+        <v>136.47</v>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
@@ -2383,25 +2376,25 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2350</v>
+        <v>2250</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>3.46</v>
+        <v>0.89</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>25.8</v>
+        <v>62.8</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>DOWNTREND 🔴</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -2410,16 +2403,16 @@
         </is>
       </c>
       <c r="K7" s="3" t="n">
-        <v>19.4</v>
+        <v>16.9</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>23.7</v>
+        <v>20.6</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>120.99</v>
+        <v>133.31</v>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
@@ -2444,16 +2437,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>26600</v>
+        <v>29100</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1.79</v>
+        <v>1.36</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>43.9</v>
+        <v>46.8</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -2471,16 +2464,16 @@
         </is>
       </c>
       <c r="K8" s="3" t="n">
-        <v>11.8</v>
+        <v>10.6</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>17.1</v>
+        <v>15.4</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>2261.94</v>
+        <v>2741.38</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
@@ -2505,16 +2498,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>21550</v>
+        <v>22200</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.03</v>
+        <v>-2.73</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>63</v>
+        <v>51.9</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -2532,16 +2525,16 @@
         </is>
       </c>
       <c r="K9" s="3" t="n">
-        <v>17</v>
+        <v>17.6</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>20.8</v>
+        <v>21.5</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>1265.96</v>
+        <v>1261.29</v>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
@@ -2566,16 +2559,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>11550</v>
+        <v>11050</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-2.61</v>
+        <v>-2.44</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>-0.02</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>53.2</v>
+        <v>48</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -2593,16 +2586,16 @@
         </is>
       </c>
       <c r="K10" s="3" t="n">
-        <v>21.7</v>
+        <v>20.5</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>20.7</v>
+        <v>19.5</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>531.05</v>
+        <v>537.75</v>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
@@ -2627,16 +2620,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>5950</v>
+        <v>6850</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1.33</v>
+        <v>2.72</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>57</v>
+        <v>52.7</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
@@ -2654,16 +2647,16 @@
         </is>
       </c>
       <c r="K11" s="3" t="n">
-        <v>19.8</v>
+        <v>22</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>18.8</v>
+        <v>20.9</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>299.91</v>
+        <v>311.59</v>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
@@ -2691,13 +2684,13 @@
         <v>1950</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.91</v>
+        <v>-0.89</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>-0.05</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>43.7</v>
+        <v>47.7</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -2715,16 +2708,16 @@
         </is>
       </c>
       <c r="K12" s="3" t="n">
-        <v>30.6</v>
+        <v>29.2</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>21.8</v>
+        <v>20.9</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>63.76</v>
+        <v>66.67</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
@@ -2749,16 +2742,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3250</v>
+        <v>3300</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1.03</v>
+        <v>-2.69</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>47.9</v>
+        <v>39.2</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -2776,16 +2769,16 @@
         </is>
       </c>
       <c r="K13" s="3" t="n">
-        <v>29.1</v>
+        <v>27.1</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>20.8</v>
+        <v>19.4</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>111.87</v>
+        <v>121.67</v>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
@@ -2810,16 +2803,16 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>62150</v>
+        <v>54150</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>-1.6</v>
+        <v>2.97</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0</v>
+        <v>0.01</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>40.5</v>
+        <v>47.3</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -2837,16 +2830,16 @@
         </is>
       </c>
       <c r="K14" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>12.5</v>
+        <v>12.8</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>7476.47</v>
+        <v>6359.42</v>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
@@ -2874,13 +2867,13 @@
         <v>1350</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.41</v>
+        <v>-0.01</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>56.2</v>
+        <v>49.8</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -2898,16 +2891,16 @@
         </is>
       </c>
       <c r="K15" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>1.2</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>12.5</v>
+        <v>11.7</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>162.58</v>
+        <v>172.37</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
@@ -2932,16 +2925,16 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7550</v>
+        <v>7400</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>-0.63</v>
+        <v>0.19</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>55.5</v>
+        <v>58.2</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
@@ -2959,16 +2952,16 @@
         </is>
       </c>
       <c r="K16" s="3" t="n">
-        <v>14.3</v>
+        <v>15</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>14.3</v>
+        <v>15</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>528.01</v>
+        <v>494.06</v>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
@@ -2993,16 +2986,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>6250</v>
+        <v>5800</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>-2.52</v>
+        <v>2.85</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>-0.04</v>
+        <v>0.05</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>53.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
@@ -3020,16 +3013,16 @@
         </is>
       </c>
       <c r="K17" s="3" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
       <c r="L17" s="3" t="n">
         <v>2.1</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>393.32</v>
+        <v>360.6</v>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
@@ -3054,16 +3047,16 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>8050</v>
+        <v>9000</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>2.22</v>
+        <v>1.19</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>51</v>
+        <v>56.4</v>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
@@ -3081,16 +3074,16 @@
         </is>
       </c>
       <c r="K18" s="3" t="n">
-        <v>15.4</v>
+        <v>15.2</v>
       </c>
       <c r="L18" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>15.4</v>
+        <v>15.2</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>523.8200000000001</v>
+        <v>592.42</v>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
@@ -3115,16 +3108,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4250</v>
+        <v>4600</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-2.69</v>
+        <v>-2.97</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>-0.06</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>48.8</v>
+        <v>32.9</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
@@ -3136,22 +3129,22 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K19" s="3" t="n">
-        <v>15.7</v>
+        <v>14.4</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>10.5</v>
+        <v>9.6</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>270.82</v>
+        <v>319.21</v>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
@@ -3176,16 +3169,16 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1150</v>
+        <v>1200</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2.81</v>
+        <v>2.95</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>49.7</v>
+        <v>43.9</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
@@ -3203,16 +3196,16 @@
         </is>
       </c>
       <c r="K20" s="3" t="n">
-        <v>15.2</v>
+        <v>16</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>15.2</v>
+        <v>16</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>75.70999999999999</v>
+        <v>75.14</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -3237,16 +3230,16 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>16150</v>
+        <v>14950</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>51.9</v>
+        <v>42.7</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
@@ -3264,16 +3257,16 @@
         </is>
       </c>
       <c r="K21" s="3" t="n">
-        <v>8.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>12.2</v>
+        <v>13</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>1991.51</v>
+        <v>1721.59</v>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
@@ -3366,25 +3359,25 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>9658</v>
+        <v>9441</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9769.82</v>
+        <v>9743.610000000001</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9932.200000000001</v>
+        <v>9832.48</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>197851.59</v>
+        <v>195048.75</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>51.6</v>
+        <v>37.2</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>9300</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10300</v>
+        <v>10200</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
@@ -3404,19 +3397,19 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>4772</v>
+        <v>5035</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>4883.03</v>
+        <v>4887.78</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>4882.44</v>
+        <v>4820</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>97012.84</v>
+        <v>95247.33</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>39.2</v>
+        <v>68</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>4500</v>
@@ -3442,19 +3435,19 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3107</v>
+        <v>3014</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>3071.93</v>
+        <v>3030.59</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3071.89</v>
+        <v>3070.64</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>61866.63</v>
+        <v>61933.89</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>55.2</v>
+        <v>56.7</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>2900</v>
@@ -3480,25 +3473,25 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>5728</v>
+        <v>5674</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5894.68</v>
+        <v>5742.59</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5846.89</v>
+        <v>5749.94</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>116871.91</v>
+        <v>115764.41</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>55.5</v>
+        <v>61.3</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>5600</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>6200</v>
+        <v>5900</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
@@ -3518,25 +3511,25 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>3610</v>
+        <v>3470</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>3541.69</v>
+        <v>3586.75</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3559.27</v>
+        <v>3595.24</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>71804.59</v>
+        <v>71729.66</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>60.2</v>
+        <v>62.1</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>3400</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>3700</v>
+        <v>3800</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
@@ -3556,25 +3549,25 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2317</v>
+        <v>2311</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2333.95</v>
+        <v>2385.12</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2343.56</v>
+        <v>2430.05</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>47522.07</v>
+        <v>48182.2</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>40.6</v>
+        <v>44.3</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>2300</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>2500</v>
+        <v>2600</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
@@ -3594,22 +3587,22 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>28231</v>
+        <v>28263</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>27062.01</v>
+        <v>27171.56</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>27198.57</v>
+        <v>26827.1</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>542754.05</v>
+        <v>537495.33</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>52.6</v>
+        <v>54.7</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>25300</v>
+        <v>25400</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>28800</v>
@@ -3632,25 +3625,25 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>20270</v>
+        <v>20778</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>20868.34</v>
+        <v>21181.53</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>21176.12</v>
+        <v>20788.21</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>422668.51</v>
+        <v>421202.21</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>61.6</v>
+        <v>54.6</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>19900</v>
+        <v>20400</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>22000</v>
+        <v>22300</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
@@ -3670,25 +3663,25 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>9773</v>
+        <v>10224</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>10052.26</v>
+        <v>10194.14</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>10129.13</v>
+        <v>10143.81</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>203767.97</v>
+        <v>203904.34</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>54.9</v>
+        <v>43.2</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>9600</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>10700</v>
+        <v>10800</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
@@ -3708,25 +3701,25 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>6585</v>
+        <v>7122</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>6690.52</v>
+        <v>6859.46</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>6745.98</v>
+        <v>6867.43</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>135956.92</v>
+        <v>138072.2</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>36</v>
+        <v>51.8</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>6400</v>
+        <v>6300</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>7000</v>
+        <v>7300</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
@@ -3746,19 +3739,19 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1727</v>
+        <v>1732</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1722.19</v>
+        <v>1727.47</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1727.41</v>
+        <v>1708.57</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>34388.5</v>
+        <v>34351.28</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>65.5</v>
+        <v>54.6</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>1600</v>
@@ -3784,25 +3777,25 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>3066</v>
+        <v>3125</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3066.99</v>
+        <v>3126.21</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3076.58</v>
+        <v>3118.03</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>61812.82</v>
+        <v>62212.84</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>50.9</v>
+        <v>59.3</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>2900</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>3200</v>
+        <v>3300</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
@@ -3822,25 +3815,25 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>55979</v>
+        <v>56126</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>56551.29</v>
+        <v>57123.93</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>57243.32</v>
+        <v>57230.73</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>1154333.57</v>
+        <v>1156014.33</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>51</v>
+        <v>58.3</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>54200</v>
+        <v>55000</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>59900</v>
+        <v>58900</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
@@ -3860,19 +3853,19 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1357</v>
+        <v>1353</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1358.9</v>
+        <v>1332.06</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1360.59</v>
+        <v>1333.61</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>27003.38</v>
+        <v>26782.08</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>49</v>
+        <v>38.1</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>1300</v>
@@ -3898,25 +3891,25 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>8227</v>
+        <v>8755</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>8454.76</v>
+        <v>8610.139999999999</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>8488.790000000001</v>
+        <v>8551.08</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>169870.87</v>
+        <v>171453.67</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>50.1</v>
+        <v>60.2</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>8100</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>9100</v>
+        <v>8900</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
@@ -3936,25 +3929,25 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>6680</v>
+        <v>6500</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>6917.54</v>
+        <v>6846.91</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>6851.69</v>
+        <v>6825.51</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>137214.79</v>
+        <v>136337.29</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>42.6</v>
+        <v>49.5</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>6500</v>
+        <v>6400</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>7200</v>
+        <v>7300</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
@@ -3974,25 +3967,25 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>9080</v>
+        <v>9337</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>9305.15</v>
+        <v>9170.68</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>9211.07</v>
+        <v>9278.559999999999</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>184361.62</v>
+        <v>185951.54</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>47.8</v>
+        <v>49.7</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>8800</v>
+        <v>8700</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>9800</v>
+        <v>9600</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
@@ -4012,25 +4005,25 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>4734</v>
+        <v>4630</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>4682.88</v>
+        <v>4759.15</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4710.89</v>
+        <v>4789.29</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>94390.35000000001</v>
+        <v>95683.39999999999</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>44</v>
+        <v>47.3</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>4500</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>4900</v>
+        <v>5000</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
@@ -4050,19 +4043,19 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>1182</v>
+        <v>1220</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1214.26</v>
+        <v>1238.94</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1214.28</v>
+        <v>1216.87</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>23892.04</v>
+        <v>24049.33</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>59.1</v>
+        <v>47.3</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>1200</v>
@@ -4088,25 +4081,25 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>14830</v>
+        <v>13627</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>14444.12</v>
+        <v>14052.06</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>14317.67</v>
+        <v>14222.69</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>285295.35</v>
+        <v>282566.13</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>54.2</v>
+        <v>48</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>13800</v>
+        <v>13400</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>15200</v>
+        <v>15000</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
@@ -4238,32 +4231,32 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9575</v>
+        <v>9970</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>867.62</v>
+        <v>841.34</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>6940.97</v>
+        <v>6730.75</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>11</v>
+        <v>11.8</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>13.8</v>
+        <v>14.8</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>1.21</v>
+        <v>0.95</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1.35</v>
+        <v>1.49</v>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>4.7%</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -4294,32 +4287,32 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>4604</v>
+        <v>4788</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>370.53</v>
+        <v>366.47</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2964.28</v>
+        <v>2931.74</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>12.4</v>
+        <v>13.1</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>15.5</v>
+        <v>16.3</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.8</v>
+        <v>1.43</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>4.9%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -4350,32 +4343,32 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2982</v>
+        <v>3048</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>209.04</v>
+        <v>216.32</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1170.61</v>
+        <v>1211.4</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>14.3</v>
+        <v>14.1</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.44</v>
+        <v>0.21</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>1.22</v>
+        <v>1.95</v>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>3.3%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -4406,28 +4399,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5612</v>
+        <v>5743</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>576.98</v>
+        <v>615.77</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>3205.43</v>
+        <v>3420.95</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>13.6</v>
+        <v>13.1</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.39</v>
+        <v>0.32</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>1.53</v>
+        <v>1.84</v>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
@@ -4462,32 +4455,32 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3658</v>
+        <v>3733</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>144.73</v>
+        <v>137.78</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>904.54</v>
+        <v>861.1</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>25.3</v>
+        <v>27.1</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>18.2</v>
+        <v>19.5</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.28</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>1.51</v>
+        <v>1.39</v>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>1.8%</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -4518,32 +4511,32 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2299</v>
+        <v>2343</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>138.85</v>
+        <v>125.03</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>833.08</v>
+        <v>750.16</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>16.6</v>
+        <v>18.7</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>20.2</v>
+        <v>22.9</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.31</v>
+        <v>0.48</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>1.88</v>
+        <v>1.77</v>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -4574,32 +4567,32 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>27475</v>
+        <v>27385</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2698.03</v>
+        <v>2731.74</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>18548.99</v>
+        <v>18780.69</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>14.8</v>
+        <v>14.6</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.2</v>
+        <v>0.34</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>1.7</v>
+        <v>1.47</v>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>1.6%</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -4630,32 +4623,32 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>21550</v>
+        <v>20278</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1295.98</v>
+        <v>1240.55</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>7775.86</v>
+        <v>7443.28</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>16.6</v>
+        <v>16.3</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>20.3</v>
+        <v>20</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>0.25</v>
+        <v>0.34</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>1.92</v>
+        <v>1.66</v>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>2.1%</t>
+          <t>2.4%</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -4686,32 +4679,32 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>10337</v>
+        <v>10105</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>473.27</v>
+        <v>519.35</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>2704.4</v>
+        <v>2967.73</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>21.8</v>
+        <v>19.5</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>20.7</v>
+        <v>18.5</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.44</v>
+        <v>0.5</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>1.32</v>
+        <v>1.49</v>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>3.1%</t>
+          <t>3.8%</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -4742,32 +4735,32 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>6707</v>
+        <v>6563</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>315.47</v>
+        <v>334.2</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1802.71</v>
+        <v>1909.69</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>21.3</v>
+        <v>19.6</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>3.7</v>
+        <v>3.4</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>20.2</v>
+        <v>18.7</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.32</v>
+        <v>0.25</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>1.4</v>
+        <v>1.66</v>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>3.0%</t>
+          <t>2.2%</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
@@ -4798,32 +4791,32 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1707</v>
+        <v>1771</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>59.36</v>
+        <v>62.5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>369.36</v>
+        <v>388.86</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.8</v>
+        <v>28.3</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>4.6</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>20.5</v>
+        <v>20.2</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.42</v>
+        <v>0.31</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>1.72</v>
+        <v>1.43</v>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -4854,28 +4847,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3127</v>
+        <v>3214</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>106.82</v>
+        <v>123.41</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>664.65</v>
+        <v>767.87</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>29.3</v>
+        <v>26</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>20.9</v>
+        <v>18.6</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>1.48</v>
+        <v>1.53</v>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
@@ -4910,32 +4903,32 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>56887</v>
+        <v>59613</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>7224.59</v>
+        <v>7407.02</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>48163.93</v>
+        <v>49380.13</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>1.2</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>11.8</v>
+        <v>12.1</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.48</v>
+        <v>0.68</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>2.02</v>
+        <v>2.13</v>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>6.4%</t>
+          <t>8.1%</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -4966,32 +4959,32 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1386</v>
+        <v>1350</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>163.31</v>
+        <v>154.77</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1088.7</v>
+        <v>1031.83</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>8.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>1.3</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>12.7</v>
+        <v>13.1</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.71</v>
+        <v>0.67</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>1.64</v>
+        <v>2.04</v>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5022,32 +5015,32 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>8449</v>
+        <v>8500</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>615.89</v>
+        <v>537.33</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>4619.16</v>
+        <v>4029.97</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>13.7</v>
+        <v>15.8</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>13.7</v>
+        <v>15.8</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.47</v>
+        <v>0.45</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>1.48</v>
+        <v>1.85</v>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>2.3%</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -5055,9 +5048,9 @@
           <t>Large Cap</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -5078,32 +5071,32 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>7020</v>
+        <v>6863</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>439.33</v>
+        <v>456.45</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>3295.01</v>
+        <v>3423.36</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.58</v>
+        <v>0.44</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1.39</v>
+        <v>1.83</v>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2.6%</t>
+          <t>2.0%</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -5134,25 +5127,25 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>9063</v>
+        <v>9183</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>626.09</v>
+        <v>622.03</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>4695.66</v>
+        <v>4665.22</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>14.5</v>
+        <v>14.8</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>14.5</v>
+        <v>14.8</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.44</v>
+        <v>0.22</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>1.75</v>
@@ -5190,32 +5183,32 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4887</v>
+        <v>4835</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>341.86</v>
+        <v>349.83</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>2563.94</v>
+        <v>2623.71</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>14.3</v>
+        <v>13.8</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>9.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1.72</v>
+        <v>1.5</v>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>2.3%</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -5246,32 +5239,32 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1156</v>
+        <v>1233</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>85.34999999999999</v>
+        <v>88.27</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>640.15</v>
+        <v>662.04</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.39</v>
+        <v>0.43</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1.44</v>
+        <v>1.43</v>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -5302,32 +5295,32 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>14227</v>
+        <v>13638</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>1716.03</v>
+        <v>1555.57</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>11440.23</v>
+        <v>10370.46</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>12.4</v>
+        <v>13.2</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>2.11</v>
+        <v>2.38</v>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>8.0%</t>
+          <t>7.9%</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
@@ -5368,7 +5361,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
@@ -5425,7 +5418,7 @@
           <t>ANTM.JK</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Aneka Tambang</t>
         </is>
@@ -5471,7 +5464,7 @@
           <t>ICBP.JK</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Indofood CBP</t>
         </is>
@@ -5517,7 +5510,7 @@
           <t>KLBF.JK</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Kalbe Farma</t>
         </is>
@@ -5563,7 +5556,7 @@
           <t>PGAS.JK</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>PGN Gas</t>
         </is>
@@ -5609,7 +5602,7 @@
           <t>UNVR.JK</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Unilever</t>
         </is>
@@ -5655,7 +5648,7 @@
           <t>HMSP.JK</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Sampoerna</t>
         </is>
@@ -5701,7 +5694,7 @@
           <t>BBCA.JK</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>BCA</t>
         </is>
@@ -5747,7 +5740,7 @@
           <t>TLKM.JK</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Telkom</t>
         </is>
@@ -5793,7 +5786,7 @@
           <t>PTUN.JK</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Platinum</t>
         </is>
@@ -5839,7 +5832,7 @@
           <t>INTP.JK</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Indocement</t>
         </is>
@@ -5898,21 +5891,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>📊 DASHBOARD SAHAM INDONESIA</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Last Update: 2026-06-27 17:47</t>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Last Update: 2026-06-27 17:46</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>IHSG Level</t>
         </is>
@@ -5924,7 +5917,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>IHSG Change</t>
         </is>
@@ -5936,7 +5929,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Top Sector</t>
         </is>
@@ -5948,7 +5941,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Worst Sector</t>
         </is>
@@ -5960,69 +5953,69 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr"/>
+      <c r="A8" s="11" t="inlineStr"/>
       <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>BUY Signals</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>SELL Signals</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>HOLD Signals</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr"/>
+      <c r="A12" s="11" t="inlineStr"/>
       <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Best Buy Today</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>ANTM.JK, KLBF.JK, INTP.JK</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Avoid</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>UNVR.JK, HMSP.JK</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Speculative</t>
         </is>

</xml_diff>

<commit_message>
Complete rewrite sentimen_berita.py - direct news homepage scraping via Jina
</commit_message>
<xml_diff>
--- a/data/harga_saham_ihsg.xlsx
+++ b/data/harga_saham_ihsg.xlsx
@@ -561,23 +561,23 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>5788.91</v>
+        <v>5817.93</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>-11.09</v>
+        <v>17.93</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>-0.19</v>
+        <v>0.31</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>5798.96</v>
+        <v>5821.81</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>5765.79</v>
+        <v>5799.05</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>657M</t>
+          <t>630M</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -593,23 +593,23 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>5776.74</v>
+        <v>5801.58</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1.51</v>
+        <v>-2.94</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>5781.7</v>
+        <v>5822.6</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>5747.07</v>
+        <v>5792.55</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>543M</t>
+          <t>736M</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -625,28 +625,28 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>5766.02</v>
+        <v>5891.05</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>2.44</v>
+        <v>59.74</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.04</v>
+        <v>1.01</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>5776.18</v>
+        <v>5891.47</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5739.38</v>
+        <v>5861.57</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>535M</t>
+          <t>798M</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -657,28 +657,28 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>5801.38</v>
+        <v>5883.36</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>-25.52</v>
+        <v>55.92</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>-0.44</v>
+        <v>0.95</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5812.02</v>
+        <v>5890.69</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>5780.75</v>
+        <v>5860.49</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>739M</t>
+          <t>613M</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -689,23 +689,23 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>5868.83</v>
+        <v>5851.47</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>15.72</v>
+        <v>-12.85</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.27</v>
+        <v>-0.22</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>5879.8</v>
+        <v>5858.09</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>5843.9</v>
+        <v>5827.77</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>644M</t>
+          <t>513M</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -721,23 +721,23 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>5821.84</v>
+        <v>5777.23</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2.25</v>
+        <v>-5.66</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.04</v>
+        <v>-0.1</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>5824.5</v>
+        <v>5794.41</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>5806.56</v>
+        <v>5774.37</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>710M</t>
+          <t>750M</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -753,19 +753,19 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>5855.93</v>
+        <v>5852</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>-7.6</v>
+        <v>59.65</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>-0.13</v>
+        <v>1.02</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5858.88</v>
+        <v>5855.58</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5842.84</v>
+        <v>5841.33</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -774,7 +774,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -785,28 +785,28 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>5895.75</v>
+        <v>5827.76</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>48.5</v>
+        <v>-2.84</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.82</v>
+        <v>-0.05</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>5914.06</v>
+        <v>5850.19</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>5891.38</v>
+        <v>5823.83</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>551M</t>
+          <t>720M</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -817,28 +817,28 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>5800.92</v>
+        <v>5738.44</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>-48.34</v>
+        <v>14.4</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>-0.83</v>
+        <v>0.25</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>5819.44</v>
+        <v>5768.39</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>5774.65</v>
+        <v>5735.04</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>706M</t>
+          <t>637M</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -849,28 +849,28 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>5881.46</v>
+        <v>5738.34</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>-10.36</v>
+        <v>-41.78</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.18</v>
+        <v>-0.73</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5902.5</v>
+        <v>5740.1</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>5866.58</v>
+        <v>5731.82</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>522M</t>
+          <t>787M</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -881,28 +881,28 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>5861.37</v>
+        <v>5806.36</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>43.07</v>
+        <v>-31.3</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.73</v>
+        <v>-0.54</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5870.29</v>
+        <v>5806.52</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>5832.24</v>
+        <v>5805.17</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>784M</t>
+          <t>521M</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -913,28 +913,28 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>5813.4</v>
+        <v>5835.7</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>-44.42</v>
+        <v>5.11</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>-0.76</v>
+        <v>0.09</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>5813.83</v>
+        <v>5860.27</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>5803.12</v>
+        <v>5826.13</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>543M</t>
+          <t>609M</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -945,28 +945,28 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>5761.2</v>
+        <v>5991.85</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>-40.38</v>
+        <v>47.08</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>-0.7</v>
+        <v>0.79</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>5768.23</v>
+        <v>5999.94</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>5733.91</v>
+        <v>5965.98</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>603M</t>
+          <t>609M</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -977,28 +977,28 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>5917.93</v>
+        <v>5854.44</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>-18.15</v>
+        <v>-31.45</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>-0.31</v>
+        <v>-0.54</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>5927.21</v>
+        <v>5881.18</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>5888.94</v>
+        <v>5849.81</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>588M</t>
+          <t>559M</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1009,23 +1009,23 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>5971.99</v>
+        <v>5882.17</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>30.78</v>
+        <v>43.14</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.52</v>
+        <v>0.73</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>5988.79</v>
+        <v>5902.2</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>5952.73</v>
+        <v>5855.72</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>672M</t>
+          <t>724M</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1041,28 +1041,28 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>5820.73</v>
+        <v>5969.18</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>-18.34</v>
+        <v>50.18</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>-0.32</v>
+        <v>0.84</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>5844.5</v>
+        <v>5972.42</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>5807.07</v>
+        <v>5942.38</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>697M</t>
+          <t>688M</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1073,28 +1073,28 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>5882.81</v>
+        <v>5949.55</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>43.16</v>
+        <v>-21.93</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.73</v>
+        <v>-0.37</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>5905.41</v>
+        <v>5972.39</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>5863.16</v>
+        <v>5945.88</v>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>580M</t>
+          <t>786M</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1105,28 +1105,28 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>5899.53</v>
+        <v>5804.19</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>55.41</v>
+        <v>15.34</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.26</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>5925.12</v>
+        <v>5820.47</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>5891.85</v>
+        <v>5797.3</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>735M</t>
+          <t>720M</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1137,28 +1137,28 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>5816.7</v>
+        <v>5990.91</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>19.85</v>
+        <v>39.01</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.34</v>
+        <v>0.65</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>5845.56</v>
+        <v>6020.35</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>5790.09</v>
+        <v>5977.08</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>689M</t>
+          <t>736M</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1169,28 +1169,28 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>5908.96</v>
+        <v>5747.29</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>-42.91</v>
+        <v>59.44</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>-0.73</v>
+        <v>1.03</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>5918.81</v>
+        <v>5775.83</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>5890.24</v>
+        <v>5737.83</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>780M</t>
+          <t>740M</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1201,19 +1201,19 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>5938.92</v>
+        <v>5705</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>28.65</v>
+        <v>-33.57</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.48</v>
+        <v>-0.59</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>5945.81</v>
+        <v>5729.52</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>5913.81</v>
+        <v>5684.66</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1233,28 +1233,28 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>5721.81</v>
+        <v>5929.76</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>-36.49</v>
+        <v>59.34</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.64</v>
+        <v>1</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>5743.9</v>
+        <v>5941.38</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>5700.58</v>
+        <v>5904.72</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>776M</t>
+          <t>672M</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Negatif</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1265,28 +1265,28 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>5828.96</v>
+        <v>5646.79</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>21.39</v>
+        <v>-20.72</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.37</v>
+        <v>-0.37</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>5842</v>
+        <v>5673.54</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5809.84</v>
+        <v>5630.83</v>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>679M</t>
+          <t>540M</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1297,28 +1297,28 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>5764.81</v>
+        <v>5876.55</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>-6.37</v>
+        <v>-25.12</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>-0.11</v>
+        <v>-0.43</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>5788.33</v>
+        <v>5883.18</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>5752.05</v>
+        <v>5855.76</v>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>728M</t>
+          <t>558M</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1329,28 +1329,28 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>5964.13</v>
+        <v>5990.59</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>43.3</v>
+        <v>-16.26</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.73</v>
+        <v>-0.27</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>5993.63</v>
+        <v>6016.66</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>5935.9</v>
+        <v>5973.38</v>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>751M</t>
+          <t>778M</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Positif</t>
+          <t>Netral</t>
         </is>
       </c>
     </row>
@@ -1361,28 +1361,28 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>5761.85</v>
+        <v>6051.74</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>-18.51</v>
+        <v>35.95</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.32</v>
+        <v>0.59</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>5780.05</v>
+        <v>6079.61</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>5749.62</v>
+        <v>6042.69</v>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>681M</t>
+          <t>701M</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Positif</t>
         </is>
       </c>
     </row>
@@ -1393,28 +1393,28 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>5886.57</v>
+        <v>5601.18</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>6.53</v>
+        <v>-35.79</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0.11</v>
+        <v>-0.64</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>5887.45</v>
+        <v>5606.39</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>5885.72</v>
+        <v>5575.03</v>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>524M</t>
+          <t>556M</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1425,28 +1425,28 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>5832.26</v>
+        <v>5575.81</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>9.210000000000001</v>
+        <v>-47.23</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.16</v>
+        <v>-0.85</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>5841.91</v>
+        <v>5576.67</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>5816</v>
+        <v>5574.26</v>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>609M</t>
+          <t>538M</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1457,23 +1457,23 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>5825.63</v>
+        <v>5909.22</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>41.81</v>
+        <v>54.33</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>5851.21</v>
+        <v>5915.17</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>5824.49</v>
+        <v>5898.43</v>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>724M</t>
+          <t>628M</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -1489,28 +1489,28 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>5870.92</v>
+        <v>5753.73</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>15.9</v>
+        <v>-20.48</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.27</v>
+        <v>-0.36</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>5896.84</v>
+        <v>5769.66</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>5843.84</v>
+        <v>5728.73</v>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>563M</t>
+          <t>662M</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Netral</t>
+          <t>Negatif</t>
         </is>
       </c>
     </row>
@@ -1521,23 +1521,23 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>5936.66</v>
+        <v>5849.15</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>18.95</v>
+        <v>-13.48</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.32</v>
+        <v>-0.23</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>5947.6</v>
+        <v>5850.24</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>5912.04</v>
+        <v>5826.34</v>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>640M</t>
+          <t>638M</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -2071,16 +2071,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10050</v>
+        <v>9000</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1.58</v>
+        <v>-2.1</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.02</v>
+        <v>-0.02</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>47.6</v>
+        <v>49.1</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
@@ -2098,16 +2098,16 @@
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v>11</v>
+        <v>11.1</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>1.4</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>917.05</v>
+        <v>808.21</v>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
@@ -2132,16 +2132,16 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>4150</v>
+        <v>5250</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>-0.48</v>
+        <v>3.82</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>-0.01</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>40.1</v>
+        <v>49.1</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
@@ -2159,16 +2159,16 @@
         </is>
       </c>
       <c r="K3" s="3" t="n">
-        <v>12.5</v>
+        <v>11.6</v>
       </c>
       <c r="L3" s="3" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>15.6</v>
+        <v>14.5</v>
       </c>
       <c r="N3" s="3" t="n">
-        <v>333.19</v>
+        <v>451.08</v>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
@@ -2193,16 +2193,16 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2900</v>
+        <v>2750</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>-0.73</v>
+        <v>3.63</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>-0.03</v>
+        <v>0.13</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>48.4</v>
+        <v>39</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -2214,22 +2214,22 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="K4" s="3" t="n">
-        <v>13.6</v>
+        <v>15.1</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>16.6</v>
+        <v>18.4</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>212.65</v>
+        <v>181.6</v>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
@@ -2254,16 +2254,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5750</v>
+        <v>5250</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>-0.03</v>
+        <v>3.01</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>-0</v>
+        <v>0.06</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>51.3</v>
+        <v>41</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -2281,16 +2281,16 @@
         </is>
       </c>
       <c r="K5" s="3" t="n">
-        <v>10.7</v>
+        <v>9.9</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>15</v>
+        <v>13.8</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>535.17</v>
+        <v>531.65</v>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
@@ -2315,16 +2315,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3500</v>
+        <v>3800</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1.12</v>
+        <v>-2.57</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.03</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>45.5</v>
+        <v>66</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -2342,16 +2342,16 @@
         </is>
       </c>
       <c r="K6" s="3" t="n">
-        <v>25.6</v>
+        <v>24.7</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>18.5</v>
+        <v>17.8</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>136.47</v>
+        <v>153.76</v>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
@@ -2376,16 +2376,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2250</v>
+        <v>2200</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.89</v>
+        <v>-2.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.04</v>
+        <v>-0.13</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>62.8</v>
+        <v>59.5</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
         </is>
       </c>
       <c r="K7" s="3" t="n">
-        <v>16.9</v>
+        <v>18.2</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>20.6</v>
+        <v>22.3</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>133.31</v>
+        <v>120.78</v>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
@@ -2437,16 +2437,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>29100</v>
+        <v>27100</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1.36</v>
+        <v>3.94</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>46.8</v>
+        <v>49</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -2464,16 +2464,16 @@
         </is>
       </c>
       <c r="K8" s="3" t="n">
-        <v>10.6</v>
+        <v>10</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>15.4</v>
+        <v>14.6</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>2741.38</v>
+        <v>2698.81</v>
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
@@ -2498,16 +2498,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>22200</v>
+        <v>22450</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>-2.73</v>
+        <v>1.26</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>51.9</v>
+        <v>51.8</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
@@ -2525,16 +2525,16 @@
         </is>
       </c>
       <c r="K9" s="3" t="n">
-        <v>17.6</v>
+        <v>17.5</v>
       </c>
       <c r="L9" s="3" t="n">
         <v>2.9</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>1261.29</v>
+        <v>1285.19</v>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
@@ -2559,16 +2559,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>11050</v>
+        <v>9850</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>-2.44</v>
+        <v>0.51</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>-0.02</v>
+        <v>0.01</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>48</v>
+        <v>50.8</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -2586,16 +2586,16 @@
         </is>
       </c>
       <c r="K10" s="3" t="n">
-        <v>20.5</v>
+        <v>21.3</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>19.5</v>
+        <v>20.2</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>537.75</v>
+        <v>462.53</v>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
@@ -2620,16 +2620,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>6850</v>
+        <v>5900</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2.72</v>
+        <v>-1.69</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.04</v>
+        <v>-0.03</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
@@ -2647,16 +2647,16 @@
         </is>
       </c>
       <c r="K11" s="3" t="n">
-        <v>22</v>
+        <v>18.8</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>20.9</v>
+        <v>17.8</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>311.59</v>
+        <v>314.56</v>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
@@ -2681,16 +2681,16 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1950</v>
+        <v>1500</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>-0.89</v>
+        <v>-1.44</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>47.7</v>
+        <v>61.2</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -2708,16 +2708,16 @@
         </is>
       </c>
       <c r="K12" s="3" t="n">
-        <v>29.2</v>
+        <v>26.2</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>4.7</v>
+        <v>4.2</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>20.9</v>
+        <v>18.7</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>66.67</v>
+        <v>57.29</v>
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
@@ -2742,16 +2742,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3300</v>
+        <v>2700</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>-2.69</v>
+        <v>0.27</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.08</v>
+        <v>0.01</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>39.2</v>
+        <v>50</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -2769,16 +2769,16 @@
         </is>
       </c>
       <c r="K13" s="3" t="n">
-        <v>27.1</v>
+        <v>26.3</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>19.4</v>
+        <v>18.8</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>121.67</v>
+        <v>102.57</v>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
@@ -2803,16 +2803,16 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>54150</v>
+        <v>51850</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>2.97</v>
+        <v>-0.25</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.01</v>
+        <v>-0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>47.3</v>
+        <v>53.6</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -2830,16 +2830,16 @@
         </is>
       </c>
       <c r="K14" s="3" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="L14" s="3" t="n">
         <v>1.3</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>6359.42</v>
+        <v>6137.78</v>
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
@@ -2864,16 +2864,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>-0.01</v>
+        <v>1.44</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>49.8</v>
+        <v>49.2</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -2891,16 +2891,16 @@
         </is>
       </c>
       <c r="K15" s="3" t="n">
-        <v>7.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="L15" s="3" t="n">
         <v>1.2</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>11.7</v>
+        <v>12.4</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>172.37</v>
+        <v>169.41</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
@@ -2925,16 +2925,16 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>7400</v>
+        <v>9250</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.19</v>
+        <v>0.79</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>58.2</v>
+        <v>46.4</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
@@ -2946,22 +2946,22 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="K16" s="3" t="n">
-        <v>15</v>
+        <v>16.3</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>15</v>
+        <v>16.3</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>494.06</v>
+        <v>566.84</v>
       </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
@@ -2986,16 +2986,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>5800</v>
+        <v>6200</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2.85</v>
+        <v>0.05</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>64.09999999999999</v>
+        <v>39.3</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
@@ -3007,22 +3007,22 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K17" s="3" t="n">
-        <v>16.1</v>
+        <v>14.8</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>16.1</v>
+        <v>14.8</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>360.6</v>
+        <v>420.15</v>
       </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
@@ -3047,16 +3047,16 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>9000</v>
+        <v>9600</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>1.19</v>
+        <v>-1.59</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.01</v>
+        <v>-0.02</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>56.4</v>
+        <v>43.7</v>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
@@ -3068,22 +3068,22 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K18" s="3" t="n">
-        <v>15.2</v>
+        <v>13.5</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>15.2</v>
+        <v>13.5</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>592.42</v>
+        <v>708.8200000000001</v>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
@@ -3108,16 +3108,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4600</v>
+        <v>5450</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>-2.97</v>
+        <v>2.59</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>-0.06</v>
+        <v>0.05</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>32.9</v>
+        <v>39.4</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
@@ -3135,16 +3135,16 @@
         </is>
       </c>
       <c r="K19" s="3" t="n">
-        <v>14.4</v>
+        <v>13.6</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>9.6</v>
+        <v>9</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>319.21</v>
+        <v>401.62</v>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
@@ -3169,16 +3169,16 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1200</v>
+        <v>1050</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2.95</v>
+        <v>2.72</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>43.9</v>
+        <v>44.5</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
@@ -3190,22 +3190,22 @@
           <t>HOLD</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
       <c r="K20" s="3" t="n">
-        <v>16</v>
+        <v>14.1</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>16</v>
+        <v>14.1</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>75.14</v>
+        <v>74.67</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
@@ -3230,16 +3230,16 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>14950</v>
+        <v>13900</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.29</v>
+        <v>-1.73</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>42.7</v>
+        <v>51.5</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
@@ -3257,16 +3257,16 @@
         </is>
       </c>
       <c r="K21" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>1.3</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>13</v>
+        <v>12.8</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>1721.59</v>
+        <v>1632.92</v>
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
@@ -3359,25 +3359,25 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>9441</v>
+        <v>9570</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>9743.610000000001</v>
+        <v>9830.120000000001</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9832.48</v>
+        <v>9838.959999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>195048.75</v>
+        <v>195438.7</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>37.2</v>
+        <v>57</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>9300</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10200</v>
+        <v>10400</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
@@ -3397,22 +3397,22 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>5035</v>
+        <v>4699</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>4887.78</v>
+        <v>4831.92</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>4820</v>
+        <v>4802.28</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>95247.33</v>
+        <v>96294.98</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>68</v>
+        <v>66.7</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>4500</v>
+        <v>4600</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>5100</v>
@@ -3435,25 +3435,25 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3014</v>
+        <v>2957</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>3030.59</v>
+        <v>3136.4</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3070.64</v>
+        <v>3143.03</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>61933.89</v>
+        <v>62697.62</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>56.7</v>
+        <v>49</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>2900</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3200</v>
+        <v>3300</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
@@ -3473,25 +3473,25 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>5674</v>
+        <v>6024</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5742.59</v>
+        <v>6059.81</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5749.94</v>
+        <v>5949.55</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>115764.41</v>
+        <v>116955.77</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>61.3</v>
+        <v>42.3</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>5600</v>
+        <v>5900</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>5900</v>
+        <v>6200</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
@@ -3511,19 +3511,19 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>3470</v>
+        <v>3435</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>3586.75</v>
+        <v>3604.74</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3595.24</v>
+        <v>3588.36</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>71729.66</v>
+        <v>72286.98</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>62.1</v>
+        <v>58.5</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>3400</v>
@@ -3549,19 +3549,19 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2311</v>
+        <v>2516</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2385.12</v>
+        <v>2382.78</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2430.05</v>
+        <v>2416.25</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>48182.2</v>
+        <v>48637.74</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>44.3</v>
+        <v>45.5</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>2300</v>
@@ -3587,25 +3587,25 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>28263</v>
+        <v>28179</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>27171.56</v>
+        <v>27374.8</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>26827.1</v>
+        <v>27311.34</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>537495.33</v>
+        <v>540111.1899999999</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>54.7</v>
+        <v>49.7</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>25400</v>
+        <v>25800</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>28800</v>
+        <v>28700</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
@@ -3625,25 +3625,25 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>20778</v>
+        <v>20492</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>21181.53</v>
+        <v>21004.26</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>20788.21</v>
+        <v>21137.9</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>421202.21</v>
+        <v>418823.92</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>54.6</v>
+        <v>41.6</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>20400</v>
+        <v>20000</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>22300</v>
+        <v>22400</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
@@ -3663,25 +3663,25 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>10224</v>
+        <v>10275</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>10194.14</v>
+        <v>10208.64</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>10143.81</v>
+        <v>10259.49</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>203904.34</v>
+        <v>203789.76</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>43.2</v>
+        <v>52.8</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>9600</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>10800</v>
+        <v>10600</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
@@ -3701,22 +3701,22 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>7122</v>
+        <v>7130</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>6859.46</v>
+        <v>6929.85</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>6867.43</v>
+        <v>6857.38</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>138072.2</v>
+        <v>135911.18</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>51.8</v>
+        <v>52.8</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>6300</v>
+        <v>6600</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>7300</v>
@@ -3739,19 +3739,19 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>1732</v>
+        <v>1702</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1727.47</v>
+        <v>1686.21</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1708.57</v>
+        <v>1711.77</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>34351.28</v>
+        <v>34135.08</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>54.6</v>
+        <v>39.3</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>1600</v>
@@ -3777,22 +3777,22 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>3125</v>
+        <v>3024</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3126.21</v>
+        <v>3133.12</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3118.03</v>
+        <v>3111.62</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>62212.84</v>
+        <v>62289.99</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>59.3</v>
+        <v>51.9</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>2900</v>
+        <v>3000</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>3300</v>
@@ -3815,25 +3815,25 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>56126</v>
+        <v>60840</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>57123.93</v>
+        <v>59465.76</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>57230.73</v>
+        <v>58806.42</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>1156014.33</v>
+        <v>1163321.46</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>58.3</v>
+        <v>52</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>55000</v>
+        <v>55900</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>58900</v>
+        <v>62100</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
@@ -3853,19 +3853,19 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1353</v>
+        <v>1307</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1332.06</v>
+        <v>1350.77</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1333.61</v>
+        <v>1351.19</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>26782.08</v>
+        <v>27189.18</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>38.1</v>
+        <v>51.3</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>1300</v>
@@ -3891,25 +3891,25 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>8755</v>
+        <v>8844</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>8610.139999999999</v>
+        <v>8562.01</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>8551.08</v>
+        <v>8519.129999999999</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>171453.67</v>
+        <v>170640.41</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>60.2</v>
+        <v>49.3</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>8100</v>
+        <v>8000</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>8900</v>
+        <v>9000</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
@@ -3929,25 +3929,25 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
+        <v>6629</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>6790.36</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>6784.44</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>135929.43</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" s="3" t="n">
         <v>6500</v>
       </c>
-      <c r="C17" s="3" t="n">
-        <v>6846.91</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>6825.51</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>136337.29</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>6400</v>
-      </c>
       <c r="H17" s="3" t="n">
-        <v>7300</v>
+        <v>7200</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
@@ -3967,25 +3967,25 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>9337</v>
+        <v>9574</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>9170.68</v>
+        <v>9281.16</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>9278.559999999999</v>
+        <v>9257.33</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>185951.54</v>
+        <v>184475.36</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>49.7</v>
+        <v>57.1</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>8700</v>
+        <v>8800</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>9600</v>
+        <v>9800</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
@@ -4005,25 +4005,25 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>4630</v>
+        <v>4825</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>4759.15</v>
+        <v>4805.78</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4789.29</v>
+        <v>4765.36</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>95683.39999999999</v>
+        <v>95060.44</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>47.3</v>
+        <v>56.5</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>4500</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>5000</v>
+        <v>5100</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
@@ -4043,22 +4043,22 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>1220</v>
+        <v>1167</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1238.94</v>
+        <v>1192.69</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1216.87</v>
+        <v>1203.7</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>24049.33</v>
+        <v>24060.54</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>47.3</v>
+        <v>44.4</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>1300</v>
@@ -4081,25 +4081,25 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>13627</v>
+        <v>14006</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>14052.06</v>
+        <v>14228.78</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>14222.69</v>
+        <v>14258.35</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>282566.13</v>
+        <v>284563.47</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>48</v>
+        <v>51.3</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>13400</v>
+        <v>13600</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>15000</v>
+        <v>14900</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
@@ -4231,32 +4231,32 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>9970</v>
+        <v>9596</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>841.34</v>
+        <v>745.41</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>6730.75</v>
+        <v>5963.28</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>11.8</v>
+        <v>12.9</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>14.8</v>
+        <v>16.1</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.95</v>
+        <v>1.33</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1.49</v>
+        <v>1.3</v>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>4.7%</t>
+          <t>5.6%</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -4287,32 +4287,32 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>4788</v>
+        <v>4589</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>366.47</v>
+        <v>421.67</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2931.74</v>
+        <v>3373.35</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>13.1</v>
+        <v>10.9</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>16.3</v>
+        <v>13.6</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>1.43</v>
+        <v>0.55</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>1.13</v>
+        <v>1.49</v>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>3.3%</t>
+          <t>4.1%</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -4343,32 +4343,32 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>3048</v>
+        <v>3122</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>216.32</v>
+        <v>226.77</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1211.4</v>
+        <v>1269.91</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>14.1</v>
+        <v>13.8</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>17.1</v>
+        <v>16.7</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>1.95</v>
+        <v>1.48</v>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>2.4%</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -4399,13 +4399,13 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5743</v>
+        <v>5874</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>615.77</v>
+        <v>634.4400000000001</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>3420.95</v>
+        <v>3524.69</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>9.300000000000001</v>
@@ -4414,17 +4414,17 @@
         <v>1.7</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>13.1</v>
+        <v>13</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>1.84</v>
+        <v>1.93</v>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>2.8%</t>
+          <t>2.3%</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -4455,32 +4455,32 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>3733</v>
+        <v>3586</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>137.78</v>
+        <v>145.04</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>861.1</v>
+        <v>906.52</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>27.1</v>
+        <v>24.7</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>19.5</v>
+        <v>17.8</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>1.39</v>
+        <v>1.35</v>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>1.8%</t>
+          <t>2.5%</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -4511,32 +4511,32 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2343</v>
+        <v>2311</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>125.03</v>
+        <v>141.24</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>750.16</v>
+        <v>847.41</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>18.7</v>
+        <v>16.4</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>22.9</v>
+        <v>20</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>0.48</v>
+        <v>0.4</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>1.77</v>
+        <v>1.68</v>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -4567,32 +4567,32 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>27385</v>
+        <v>26411</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2731.74</v>
+        <v>2341.52</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>18780.69</v>
+        <v>16097.94</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>10</v>
+        <v>11.3</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>14.6</v>
+        <v>16.4</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.34</v>
+        <v>0.45</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>1.47</v>
+        <v>1.83</v>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>1.6%</t>
+          <t>3.1%</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -4623,32 +4623,32 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>20278</v>
+        <v>20143</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1240.55</v>
+        <v>1157.6</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>7443.28</v>
+        <v>6945.62</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>16.3</v>
+        <v>17.4</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>20</v>
+        <v>21.3</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>0.34</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>1.66</v>
+        <v>1.57</v>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>2.4%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -4679,32 +4679,32 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>10105</v>
+        <v>10043</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>519.35</v>
+        <v>511.38</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>2967.73</v>
+        <v>2922.19</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>19.5</v>
+        <v>19.6</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>3.4</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>18.5</v>
+        <v>18.7</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>1.49</v>
+        <v>1.3</v>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -4735,32 +4735,32 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>6563</v>
+        <v>6811</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>334.2</v>
+        <v>323.69</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1909.69</v>
+        <v>1849.68</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>19.6</v>
+        <v>21</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>18.7</v>
+        <v>20</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>0.25</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>1.66</v>
+        <v>1.72</v>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>2.2%</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
@@ -4791,32 +4791,32 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1771</v>
+        <v>1659</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>62.5</v>
+        <v>64.95999999999999</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>388.86</v>
+        <v>404.19</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.3</v>
+        <v>25.5</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>4.6</v>
+        <v>4.1</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>20.2</v>
+        <v>18.2</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>1.43</v>
+        <v>1.41</v>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -4847,32 +4847,32 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3214</v>
+        <v>2963</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>123.41</v>
+        <v>99.41</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>767.87</v>
+        <v>618.53</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>26</v>
+        <v>29.8</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>18.6</v>
+        <v>21.3</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>0.5</v>
+        <v>0.57</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>1.53</v>
+        <v>1.57</v>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
@@ -4903,32 +4903,32 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>59613</v>
+        <v>55417</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>7407.02</v>
+        <v>7347.79</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>49380.13</v>
+        <v>48985.24</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>0.68</v>
+        <v>0.4</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>2.13</v>
+        <v>1.88</v>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>8.1%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -4959,13 +4959,13 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1350</v>
+        <v>1388</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>154.77</v>
+        <v>159.35</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1031.83</v>
+        <v>1062.31</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>8.699999999999999</v>
@@ -4977,14 +4977,14 @@
         <v>13.1</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.67</v>
+        <v>0.31</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>8.9%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
@@ -5015,32 +5015,32 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>8500</v>
+        <v>8444</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>537.33</v>
+        <v>572.86</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>4029.97</v>
+        <v>4296.45</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>15.8</v>
+        <v>14.7</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>15.8</v>
+        <v>14.7</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>0.45</v>
+        <v>0.39</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>1.85</v>
+        <v>1.36</v>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>2.3%</t>
+          <t>1.8%</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -5048,9 +5048,9 @@
           <t>Large Cap</t>
         </is>
       </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
         </is>
       </c>
     </row>
@@ -5071,32 +5071,32 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>6863</v>
+        <v>6965</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>456.45</v>
+        <v>449.34</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>3423.36</v>
+        <v>3370.09</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>0.44</v>
+        <v>0.32</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>1.83</v>
+        <v>1.87</v>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>2.0%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
@@ -5127,32 +5127,32 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>9183</v>
+        <v>9043</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>622.03</v>
+        <v>580</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>4665.22</v>
+        <v>4350</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>14.8</v>
+        <v>15.6</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>14.8</v>
+        <v>15.6</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0.22</v>
+        <v>0.34</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1.75</v>
+        <v>1.87</v>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>3.3%</t>
+          <t>3.5%</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -5160,9 +5160,9 @@
           <t>Large Cap</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -5183,32 +5183,32 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>4835</v>
+        <v>4785</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>349.83</v>
+        <v>305.17</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>2623.71</v>
+        <v>2288.74</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>13.8</v>
+        <v>15.7</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.38</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1.5</v>
+        <v>1.31</v>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>2.3%</t>
+          <t>3.9%</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
@@ -5216,9 +5216,9 @@
           <t>Large Cap</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>BUY</t>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
@@ -5239,13 +5239,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1233</v>
+        <v>1214</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>88.27</v>
+        <v>86.56</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>662.04</v>
+        <v>649.1900000000001</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>14</v>
@@ -5257,14 +5257,14 @@
         <v>14</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>0.43</v>
+        <v>0.52</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>1.43</v>
+        <v>1.77</v>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>1.9%</t>
+          <t>2.4%</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -5295,32 +5295,32 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>13638</v>
+        <v>14699</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>1555.57</v>
+        <v>2005.77</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>10370.46</v>
+        <v>13371.83</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>13.2</v>
+        <v>11</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>0.73</v>
+        <v>0.47</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>2.38</v>
+        <v>1.95</v>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>7.9%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
@@ -5900,7 +5900,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Last Update: 2026-06-27 17:46</t>
+          <t>Last Update: 2026-06-27 20:28</t>
         </is>
       </c>
     </row>
@@ -5963,7 +5963,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -5973,7 +5973,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">

</xml_diff>